<commit_message>
Sync local workbook 2026-09-24 10:54:58
</commit_message>
<xml_diff>
--- a/data/New Import Monitoring.xlsx
+++ b/data/New Import Monitoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User-2\Dropbox\Marfani Projects\Marfani Steel Reportings\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6732E89-80D0-4B5B-A2E6-2E5B639AFE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78FF974D-6612-4261-A1D5-254367F7DDBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A600BC22-BC84-4799-95E7-AAC4792B97D7}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Compele Data Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Compele Data Sheet'!$A$3:$CV$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Compele Data Sheet'!$A$3:$CV$128</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5606" uniqueCount="1175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5620" uniqueCount="1182">
   <si>
     <t>Marfani Steel Private Limited</t>
   </si>
@@ -3706,6 +3706,27 @@
   </si>
   <si>
     <t>MOSSIMS210926691496</t>
+  </si>
+  <si>
+    <t>STAINLESS STEEL SCRAP 309 GRADE FOR MELT</t>
+  </si>
+  <si>
+    <t>SS 309</t>
+  </si>
+  <si>
+    <t>NI- 12%-15% CR- 22%-24% FE- Balance</t>
+  </si>
+  <si>
+    <t>HASU1135814</t>
+  </si>
+  <si>
+    <t>(10Jumbo Bag@4 Kg=40Kg)</t>
+  </si>
+  <si>
+    <t>JEDDAH</t>
+  </si>
+  <si>
+    <t>Jawaharlal Nehru</t>
   </si>
 </sst>
 </file>
@@ -4383,7 +4404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5597E4D-E64B-42C2-AB73-4C180426F403}">
-  <dimension ref="A1:CV127"/>
+  <dimension ref="A1:CV128"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -25878,7 +25899,7 @@
         <v>1620021365</v>
       </c>
       <c r="M70" s="13">
-        <f t="shared" ref="M70:M127" si="31">IF(AK70&gt;127000,6,IF(AK70&gt;104000, 5, IF(AK70&gt;79000, 4, IF(AK70&gt;55000, 3, IF(AK70&gt;29000, 2, IF(AK70&gt;4900, 1, 0))))))</f>
+        <f t="shared" ref="M70:M128" si="31">IF(AK70&gt;127000,6,IF(AK70&gt;104000, 5, IF(AK70&gt;79000, 4, IF(AK70&gt;55000, 3, IF(AK70&gt;29000, 2, IF(AK70&gt;4900, 1, 0))))))</f>
         <v>1</v>
       </c>
       <c r="N70" s="43">
@@ -40349,7 +40370,7 @@
         <v>735</v>
       </c>
       <c r="V123" s="24">
-        <f t="shared" ref="V123:V124" si="55">+T123*U123</f>
+        <f t="shared" ref="V123:V128" si="55">+T123*U123</f>
         <v>36750</v>
       </c>
       <c r="W123" s="24"/>
@@ -40571,7 +40592,10 @@
         <v>370</v>
       </c>
       <c r="Q125" s="17"/>
-      <c r="V125" s="24"/>
+      <c r="V125" s="24">
+        <f t="shared" si="55"/>
+        <v>0</v>
+      </c>
       <c r="W125" s="24"/>
       <c r="X125" s="24"/>
       <c r="Y125" s="28"/>
@@ -40666,7 +40690,10 @@
       <c r="R126" s="13" t="s">
         <v>1171</v>
       </c>
-      <c r="V126" s="24"/>
+      <c r="V126" s="24">
+        <f t="shared" si="55"/>
+        <v>0</v>
+      </c>
       <c r="W126" s="24"/>
       <c r="X126" s="24"/>
       <c r="Y126" s="28"/>
@@ -40750,7 +40777,10 @@
       </c>
       <c r="O127" s="16"/>
       <c r="Q127" s="17"/>
-      <c r="V127" s="24"/>
+      <c r="V127" s="24">
+        <f t="shared" si="55"/>
+        <v>0</v>
+      </c>
       <c r="W127" s="24"/>
       <c r="X127" s="24"/>
       <c r="Y127" s="28"/>
@@ -40809,7 +40839,102 @@
       </c>
       <c r="CR127" s="24"/>
     </row>
+    <row r="128" spans="1:100" s="13" customFormat="1" ht="43.2">
+      <c r="A128" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="C128" s="13" t="s">
+        <v>571</v>
+      </c>
+      <c r="D128" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E128" s="13">
+        <v>275759725</v>
+      </c>
+      <c r="F128" s="14">
+        <v>46314</v>
+      </c>
+      <c r="G128" s="14">
+        <f>F128+13</f>
+        <v>46327</v>
+      </c>
+      <c r="I128" s="15"/>
+      <c r="J128" s="15"/>
+      <c r="L128" s="13">
+        <v>1620021640</v>
+      </c>
+      <c r="M128" s="13">
+        <f t="shared" si="31"/>
+        <v>1</v>
+      </c>
+      <c r="N128" s="14">
+        <v>46268</v>
+      </c>
+      <c r="O128" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="P128" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="Q128" s="13" t="s">
+        <v>1175</v>
+      </c>
+      <c r="R128" s="13" t="s">
+        <v>1176</v>
+      </c>
+      <c r="S128" s="13" t="s">
+        <v>1177</v>
+      </c>
+      <c r="T128" s="13">
+        <v>23</v>
+      </c>
+      <c r="U128" s="13">
+        <v>2125</v>
+      </c>
+      <c r="V128" s="24">
+        <f t="shared" si="55"/>
+        <v>48875</v>
+      </c>
+      <c r="Y128" s="13">
+        <v>8110047179</v>
+      </c>
+      <c r="Z128" s="14">
+        <v>46271</v>
+      </c>
+      <c r="AA128" s="13" t="s">
+        <v>1178</v>
+      </c>
+      <c r="AB128" s="13">
+        <v>20.63</v>
+      </c>
+      <c r="AK128" s="13">
+        <v>23630</v>
+      </c>
+      <c r="AL128" s="13" t="s">
+        <v>1179</v>
+      </c>
+      <c r="AM128" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="AN128" s="13">
+        <v>26733</v>
+      </c>
+      <c r="AP128" s="13" t="s">
+        <v>1180</v>
+      </c>
+      <c r="AQ128" s="13" t="s">
+        <v>1181</v>
+      </c>
+      <c r="AR128" s="13" t="s">
+        <v>1181</v>
+      </c>
+      <c r="AS128" s="13">
+        <v>72042190</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A3:CV128" xr:uid="{E5597E4D-E64B-42C2-AB73-4C180426F403}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:CV2"/>
   </mergeCells>
@@ -40823,16 +40948,16 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA5:CA45 CA121 CA82:CA86 CA88:CA90 CA111:CA116 CA47:CA54 CA66 CA68:CA70 CA75:CA76 CA72 CA56:CA63 CA92 CA94:CA96 CA98:CA99 CA103" xr:uid="{A6F5A0E5-0F22-49D2-B71C-219719C45511}">
       <formula1>"Paid,Unpaid"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D127" xr:uid="{2D2AB97F-C76D-41DF-907F-F8CEED097798}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D128" xr:uid="{2D2AB97F-C76D-41DF-907F-F8CEED097798}">
       <formula1>"MSPL,MSI"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I122:J127 J120 I117:I120 I102 I104:I110" xr:uid="{10262EBC-1B33-427B-92F5-1FBD2FC7F498}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I104:I110 J120 I117:I120 I102 I122:J128" xr:uid="{10262EBC-1B33-427B-92F5-1FBD2FC7F498}">
       <formula1>"Surrenderred,CAD"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C127" xr:uid="{16154F91-A0D4-4BEE-AB3D-BD972A0500E1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C128" xr:uid="{16154F91-A0D4-4BEE-AB3D-BD972A0500E1}">
       <formula1>"Active,Closed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J112:J119 CH104:CH124 CH5:CH99 I112:I113 I121:J121 I111:J111 I114:J116 I103 I98:I101 I5:J97 J98:J110" xr:uid="{A0AC2255-9F46-4C74-A710-EB7A598AB0D3}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH104:CH124 CH5:CH99 J104:J119 I111:I116 I103:J103 I5:I101 J5:J102 I121:J121" xr:uid="{A0AC2255-9F46-4C74-A710-EB7A598AB0D3}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR27:AR44 AQ5:AQ20 AR22:AR25 AR52:AR55 AQ103:AR105 AQ85:AR99 AR46:AR50 AR57:AR60 AQ22:AQ84 AR62:AR84" xr:uid="{98C578F6-C2B0-46BF-BAB8-DD2E60D0AD78}">

</xml_diff>